<commit_message>
Track grade quantity and loss per consignee
Contents ending in G<n> count one item of that grade; G<n>-L<k> rows
are loss rows that add k to the grade's loss and nothing to quantity.
Adds GradeCode/LossQty columns (with an in-place upgrade for existing
databases), grade and consignee-by-grade reports with G1-G13 crosstabs,
a Consignee x grade form with Excel export, a grade list on the
dashboard, and updated sample files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sx8Nnip1bPJjGi6yYcqszE
</commit_message>
<xml_diff>
--- a/access/samples/master_inventory_sample.xlsx
+++ b/access/samples/master_inventory_sample.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EBUXSL2079602026</t>
+          <t>EBUXSL2079600001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -468,19 +468,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>نقطة توزيع المجاردة \\ G9-L1</t>
+          <t>نقطة توزيع المجاردة \\ G1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ASR-SEP30-G9</t>
+          <t>ASR-SEP30-G1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EBUXSL2079418826</t>
+          <t>EBUXSL2079600002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -490,105 +490,171 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>نقطة توزيع المجاردة \\ G9-L1</t>
+          <t>نقطة توزيع المجاردة \\ G1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ASR-SEP30-G9</t>
+          <t>ASR-SEP30-G1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EBUXSL2079500001</t>
+          <t>EBUXSL2079600003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>71205-1</t>
+          <t>71204-3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>نقطة توزيع حائل \\ G10-L2</t>
+          <t>نقطة توزيع المجاردة \\ G1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ASR-SEP30-G10</t>
+          <t>ASR-SEP30-G1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EBUXSL2079500002</t>
+          <t>EBUXSL2079600004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>71205-2</t>
+          <t>71204-4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>نقطة توزيع حائل \\ G10-L2</t>
+          <t>نقطة توزيع المجاردة \\ G1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ASR-SEP30-G10</t>
+          <t>ASR-SEP30-G1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EBUXSL2079500003</t>
+          <t>EBUXSL2079600005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>71206-1</t>
+          <t>71204-5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>نقطة توزيع أبها \\ G11-L1</t>
+          <t>نقطة توزيع المجاردة \\ G1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ASR-SEP30-G11</t>
+          <t>ASR-SEP30-G1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EBUXSL2079500004</t>
+          <t>EBUXSL2079600006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>71206-2</t>
+          <t>71204-6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>نقطة توزيع أبها \\ G11-L1</t>
+          <t>نقطة توزيع المجاردة \\ G1-L4</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ASR-SEP30-G11</t>
+          <t>ASR-SEP30-G1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EBUXSL2079700001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>71205-1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>نقطة توزيع حائل \\ G9</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ASR-SEP30-G9</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EBUXSL2079700002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>71205-2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>نقطة توزيع حائل \\ G9-L1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ASR-SEP30-G9</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EBUXSL2079700003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>71205-3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>نقطة توزيع حائل \\ G9</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ASR-SEP30-G9</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sum grade quantity and loss per master upload
Grade codes may follow \\, / or // in the contents; G<n>-L<k> counts
only as loss. Each master import now reports per-grade Qty/Loss totals
for the uploaded file, with an export button on the upload form.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sx8Nnip1bPJjGi6yYcqszE
</commit_message>
<xml_diff>
--- a/access/samples/master_inventory_sample.xlsx
+++ b/access/samples/master_inventory_sample.xlsx
@@ -600,7 +600,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>نقطة توزيع حائل \\ G9</t>
+          <t>نقطة توزيع حائل // G9</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>نقطة توزيع حائل \\ G9-L1</t>
+          <t>نقطة توزيع حائل / G9-L1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">

</xml_diff>